<commit_message>
condicion nivedu, desagregacion por edad, y script censos viejo
</commit_message>
<xml_diff>
--- a/Inputs/idef.xlsx
+++ b/Inputs/idef.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sofia\Documents\BID\2025\calculo_indicators_R\Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B75091E-F719-423D-AD8A-A0D4070DF87D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDBF4235-7DA8-4267-A656-A7544B6D625D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="10240" xr2:uid="{76C58BDB-E763-4EA4-A4AF-6A5E1AEAFFAC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{76C58BDB-E763-4EA4-A4AF-6A5E1AEAFFAC}"/>
   </bookViews>
   <sheets>
     <sheet name="idef" sheetId="1" r:id="rId1"/>
@@ -18,12 +18,25 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">idef!$A$1:$H$278</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1946" uniqueCount="675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1946" uniqueCount="676">
   <si>
     <t>indicator_name</t>
   </si>
@@ -2048,6 +2061,9 @@
   </si>
   <si>
     <t>razonesnoasis_ci == 4 &amp; edad_ci &gt;= 18 &amp; edad_ci &lt;= 24 &amp; asiste_ci != 1 &amp; nivel_edu&lt; 6</t>
+  </si>
+  <si>
+    <t>sex,age,quintile,area,ethnicity,disability,migration,isoalpha3,year</t>
   </si>
 </sst>
 </file>
@@ -2974,7 +2990,7 @@
         <v>656</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>675</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -3000,7 +3016,7 @@
         <v>660</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>675</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -3026,7 +3042,7 @@
         <v>659</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
+        <v>675</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -3052,7 +3068,7 @@
         <v>658</v>
       </c>
       <c r="F5" t="s">
-        <v>12</v>
+        <v>675</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -3754,7 +3770,7 @@
         <v>79</v>
       </c>
       <c r="F32" t="s">
-        <v>12</v>
+        <v>675</v>
       </c>
       <c r="G32" t="s">
         <v>13</v>
@@ -3780,7 +3796,7 @@
         <v>79</v>
       </c>
       <c r="F33" t="s">
-        <v>12</v>
+        <v>675</v>
       </c>
       <c r="G33" t="s">
         <v>13</v>
@@ -3806,7 +3822,7 @@
         <v>79</v>
       </c>
       <c r="F34" t="s">
-        <v>12</v>
+        <v>675</v>
       </c>
       <c r="G34" t="s">
         <v>13</v>
@@ -3832,7 +3848,7 @@
         <v>79</v>
       </c>
       <c r="F35" t="s">
-        <v>12</v>
+        <v>675</v>
       </c>
       <c r="G35" t="s">
         <v>13</v>
@@ -3858,7 +3874,7 @@
         <v>79</v>
       </c>
       <c r="F36" t="s">
-        <v>12</v>
+        <v>675</v>
       </c>
       <c r="G36" t="s">
         <v>13</v>
@@ -3884,7 +3900,7 @@
         <v>79</v>
       </c>
       <c r="F37" t="s">
-        <v>12</v>
+        <v>675</v>
       </c>
       <c r="G37" t="s">
         <v>13</v>
@@ -3910,7 +3926,7 @@
         <v>79</v>
       </c>
       <c r="F38" t="s">
-        <v>12</v>
+        <v>675</v>
       </c>
       <c r="G38" t="s">
         <v>13</v>
@@ -3936,7 +3952,7 @@
         <v>79</v>
       </c>
       <c r="F39" t="s">
-        <v>12</v>
+        <v>675</v>
       </c>
       <c r="G39" t="s">
         <v>13</v>
@@ -3962,7 +3978,7 @@
         <v>79</v>
       </c>
       <c r="F40" t="s">
-        <v>12</v>
+        <v>675</v>
       </c>
       <c r="G40" t="s">
         <v>13</v>

</xml_diff>